<commit_message>
Added Transaction Logs Module
</commit_message>
<xml_diff>
--- a/obj/Release/net8.0/PubTmp/Out/wwwroot/templates/ImportData_Batch Entry Template.xlsx
+++ b/obj/Release/net8.0/PubTmp/Out/wwwroot/templates/ImportData_Batch Entry Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caparrar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caparrar\Documents\PartsControlSystem\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14BF93A8-E2C3-40A4-A2DB-50AB77D61136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BFB74E-0A15-447E-A366-EC70B28762ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD9CB474-666E-4C8C-AA5C-D7832CB7BCFB}"/>
+    <workbookView xWindow="-28920" yWindow="-2655" windowWidth="29040" windowHeight="15720" xr2:uid="{AD9CB474-666E-4C8C-AA5C-D7832CB7BCFB}"/>
   </bookViews>
   <sheets>
     <sheet name="Batch Entry" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
   <si>
     <t>Batch Entry Template</t>
   </si>
@@ -113,6 +113,33 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Tooling Type</t>
+  </si>
+  <si>
+    <t>Tooling  Category</t>
+  </si>
+  <si>
+    <t>Injection (Tooling)</t>
+  </si>
+  <si>
+    <t>Rubber Injection (Tooling)</t>
+  </si>
+  <si>
+    <t>Stamping (Tooling)</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Additional</t>
+  </si>
+  <si>
+    <t>Renewal</t>
+  </si>
+  <si>
+    <t>New</t>
   </si>
 </sst>
 </file>
@@ -261,16 +288,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -615,7 +642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3DE9607-933D-49B1-8B31-DA028A263F67}">
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.875" customWidth="1"/>
@@ -625,24 +652,24 @@
     <col min="6" max="6" width="20.125" customWidth="1"/>
     <col min="7" max="7" width="15.375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.75" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.25" customWidth="1"/>
-    <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.75" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.25" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28" customWidth="1"/>
+    <col min="9" max="11" width="15.25" customWidth="1"/>
+    <col min="12" max="12" width="22" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="19.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="19.5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -650,86 +677,96 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="5"/>
-    </row>
-    <row r="3" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+    </row>
+    <row r="3" spans="1:20" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
       <c r="M3" s="11"/>
       <c r="N3" s="11"/>
       <c r="O3" s="11"/>
       <c r="P3" s="11"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="8" t="s">
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="3" t="s">
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="P4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="Q4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="R4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="S4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R4" s="7"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T4" s="7"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -748,8 +785,10 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -768,8 +807,10 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -788,8 +829,10 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -808,8 +851,10 @@
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -828,8 +873,10 @@
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -848,8 +895,10 @@
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -868,8 +917,10 @@
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -888,8 +939,10 @@
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -908,8 +961,10 @@
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -928,8 +983,10 @@
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -948,8 +1005,10 @@
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -968,8 +1027,10 @@
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -988,8 +1049,10 @@
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1008,8 +1071,10 @@
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1028,8 +1093,10 @@
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1048,8 +1115,10 @@
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1068,30 +1137,46 @@
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="R3:R4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="J3:Q3"/>
+  <mergeCells count="13">
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="I3:I4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="E3:E4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="L3:S3"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="K3:K4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8B88CCCE-FB45-4A85-ABDD-C6846B4B899A}">
           <x14:formula1>
             <xm:f>'Drop Down'!$E$2:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>J5:Q21</xm:sqref>
+          <xm:sqref>L5:S21</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B55F934C-214F-4C45-8854-43C6CF3CBDED}">
+          <x14:formula1>
+            <xm:f>'Drop Down'!$G$2:$G$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>J5</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8C3549AE-CCCA-4A7E-A5F7-4C8F0CA3552E}">
+          <x14:formula1>
+            <xm:f>'Drop Down'!$I$2:$I$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>K5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1101,59 +1186,92 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A66CCD1-3A7D-4468-9305-EED7289E2F78}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="22.25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
       <c r="E1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="E2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="E3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>

</xml_diff>